<commit_message>
Fix count mismatches, make Read Me counts live, tighten status drop-down
- Read Me claim totals and deadline-band counts are now formulas, which
  also corrects the June (134 -> 133) and master (477 -> 476) totals.
- Claim Status drop-down covers A2:A1000 on every specialty sheet (June
  ORTHO's last row had none), uses the same full status list in every
  file, and rejects values not on the list. Read Me wording updated.
- Removed two stray formatted empty rows below May DME's data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 00 Master v2.xlsx
+++ b/SPC26S1 - 00 Master v2.xlsx
@@ -279,7 +279,7 @@
     <t>Row order - timely filing deadline</t>
   </si>
   <si>
-    <t>Sorted the same way as the monthly workbooks: by Days Until Deadline, most urgent first, so the two views line up. A negative number means the filing window has already closed; a blank means no limit is on file. The counts below are as at 19 September 2026, and the row order is a snapshot - sort ascending on Days Until Deadline to bring it up to date.</t>
+    <t>Sorted the same way as the monthly workbooks: by Days Until Deadline, most urgent first, so the two views line up. A negative number means the filing window has already closed; a blank means no limit is on file. The counts below update automatically, and the row order is a snapshot - sort ascending on Days Until Deadline to bring it up to date.</t>
   </si>
   <si>
     <t xml:space="preserve">    1 - Due in 5 days or less: 22</t>
@@ -11753,8 +11753,9 @@
       <c r="A2" s="2"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
+      <c r="A3" s="2" t="str">
+        <f>"Every one of the "&amp;COUNTA('All Claims'!$D$2:$D$2000)&amp;" claims for 2026 S1, all specialties and all six months in one place, on the 'All Claims' tab."</f>
+        <v>Every one of the 476 claims for 2026 S1, all specialties and all six months in one place, on the 'All Claims' tab.</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -11771,28 +11772,33 @@
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>4</v>
+      <c r="A7" s="2" t="str">
+        <f>"    1 - Due in 5 days or less: "&amp;COUNTIFS('All Claims'!$L$2:$L$2000,"&gt;=0",'All Claims'!$L$2:$L$2000,"&lt;=5")</f>
+        <v>    1 - Due in 5 days or less: 1</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>5</v>
+      <c r="A8" s="2" t="str">
+        <f>"    2 - Due in 6-30 days: "&amp;COUNTIFS('All Claims'!$L$2:$L$2000,"&gt;5",'All Claims'!$L$2:$L$2000,"&lt;=30")</f>
+        <v>    2 - Due in 6-30 days: 9</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>6</v>
+      <c r="A9" s="2" t="str">
+        <f>"    3 - Due in 31+ days: "&amp;COUNTIFS('All Claims'!$L$2:$L$2000,"&gt;30")</f>
+        <v>    3 - Due in 31+ days: 149</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>7</v>
+      <c r="A10" s="2" t="str">
+        <f>"    4 - Past deadline: "&amp;COUNTIFS('All Claims'!$L$2:$L$2000,"&lt;0")</f>
+        <v>    4 - Past deadline: 274</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
+      <c r="A11" s="2" t="str">
+        <f>"    5 - No limit on file: "&amp;COUNTIFS('All Claims'!$D$2:$D$2000,"&lt;&gt;",'All Claims'!$L$2:$L$2000,"")</f>
+        <v>    5 - No limit on file: 43</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Recolor Under Review and worked Denied rows in all workbooks
Under Review rows are now bright orange with bold text so they stand
out. Denied rows keep the red only while Latest Date Worked is empty;
once a date is entered they turn light pink. Read Me legends updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 00 Master v2.xlsx
+++ b/SPC26S1 - 00 Master v2.xlsx
@@ -3504,7 +3504,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="24">
     <dxf>
       <font>
         <color rgb="FF1F4E79"/>
@@ -3687,9 +3687,13 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <color rgb="FF000000"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFFF9933"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3711,6 +3715,13 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFBFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -11738,7 +11749,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="118" customWidth="1"/>
@@ -11949,14 +11960,14 @@
     <row r="41" spans="1:1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Under Review - orange</t>
+          <t xml:space="preserve">    Under Review - bright orange, bold (follow up on these)</t>
         </is>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Denied - red</t>
+          <t xml:space="preserve">    Denied, not worked yet (Latest Date Worked empty) - red</t>
         </is>
       </c>
     </row>
@@ -11976,6 +11987,13 @@
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Denied, already worked (Latest Date Worked filled in) - light pink</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Any other status is left unshaded.</t>
         </is>
@@ -12019,6 +12037,11 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="A44">
     <cfRule type="expression" dxfId="22" priority="8">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A45">
+    <cfRule type="expression" dxfId="23" priority="9">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -69059,7 +69082,10 @@
       <formula>TRIM($A2)="Under Review"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="20" priority="21">
-      <formula>TRIM($A2)="Denied"</formula>
+      <formula>AND(TRIM($A2)="Denied",$K2="")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="24">
+      <formula>AND(TRIM($A2)="Denied",$K2&lt;&gt;"")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="21" priority="22">
       <formula>TRIM($A2)="Rejected"</formula>

</xml_diff>